<commit_message>
updated  daily routine - 11 august
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DB512CD-18D4-4733-83DB-7C914C628D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CFB383-E294-4445-A659-850020D3845F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -203,6 +203,15 @@
   </si>
   <si>
     <t>CAP776 S:D1P2631</t>
+  </si>
+  <si>
+    <t>good</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>Had a normal day</t>
   </si>
 </sst>
 </file>
@@ -984,7 +993,7 @@
     </row>
     <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
-        <v>46315</v>
+        <v>46244</v>
       </c>
       <c r="B6" s="9">
         <v>480</v>
@@ -1029,26 +1038,49 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+      <c r="A7" s="8">
+        <v>46245</v>
+      </c>
+      <c r="B7" s="14">
+        <v>480</v>
+      </c>
+      <c r="C7" s="14">
+        <v>45</v>
+      </c>
+      <c r="D7" s="14">
+        <v>120</v>
+      </c>
+      <c r="E7" s="14">
+        <v>90</v>
+      </c>
+      <c r="F7" s="14">
+        <v>180</v>
+      </c>
+      <c r="G7" s="14">
+        <v>5</v>
+      </c>
+      <c r="H7" s="14">
+        <v>60</v>
+      </c>
+      <c r="I7" s="15">
+        <v>975</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
+        <v>465</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>

</xml_diff>

<commit_message>
Updated daily routine 12 Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CFB383-E294-4445-A659-850020D3845F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E078A175-68B7-4188-BF99-C1ADA9B6FFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -212,6 +212,9 @@
   </si>
   <si>
     <t>Had a normal day</t>
+  </si>
+  <si>
+    <t>Totally Hectic day</t>
   </si>
 </sst>
 </file>
@@ -1083,26 +1086,50 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="A8" s="13">
+        <v>46246</v>
+      </c>
+      <c r="B8" s="14">
+        <v>480</v>
+      </c>
+      <c r="C8" s="14">
+        <v>45</v>
+      </c>
+      <c r="D8" s="14">
+        <v>120</v>
+      </c>
+      <c r="E8" s="14">
+        <v>90</v>
+      </c>
+      <c r="F8" s="14">
+        <v>400</v>
+      </c>
+      <c r="G8" s="14">
+        <v>8</v>
+      </c>
+      <c r="H8" s="14">
+        <v>60</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>1195</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+        <v>245</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>

</xml_diff>

<commit_message>
updated daily-routine 13 august
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E078A175-68B7-4188-BF99-C1ADA9B6FFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4046A402-2290-46AF-BFE8-AEECEF5F4E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -215,6 +215,12 @@
   </si>
   <si>
     <t>Totally Hectic day</t>
+  </si>
+  <si>
+    <t>satisfied</t>
+  </si>
+  <si>
+    <t>had a debate in communication class mam appreciated felt happy</t>
   </si>
 </sst>
 </file>
@@ -1131,27 +1137,51 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+    <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
+        <v>46247</v>
+      </c>
+      <c r="B9" s="14">
+        <v>480</v>
+      </c>
+      <c r="C9" s="14">
+        <v>45</v>
+      </c>
+      <c r="D9" s="14">
+        <v>120</v>
+      </c>
+      <c r="E9" s="14">
+        <v>90</v>
+      </c>
+      <c r="F9" s="14">
+        <v>560</v>
+      </c>
+      <c r="G9" s="14">
+        <v>7</v>
+      </c>
+      <c r="H9" s="14">
+        <v>60</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>1355</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>85</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>

</xml_diff>

<commit_message>
updated daily-routine 16- August
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4676D9-E7F0-4EEC-BF4C-CC60E9552478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DFDC80-FB2F-4B75-BB66-5CB7C97EB69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -224,6 +224,21 @@
   </si>
   <si>
     <t>had a normal day</t>
+  </si>
+  <si>
+    <t>relaxed</t>
+  </si>
+  <si>
+    <t>watched a lecture of networking feeling great</t>
+  </si>
+  <si>
+    <t>neutral</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">had a normal day </t>
   </si>
 </sst>
 </file>
@@ -1232,49 +1247,97 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>46249</v>
+      </c>
+      <c r="B11" s="14">
+        <v>600</v>
+      </c>
+      <c r="C11" s="14">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14">
+        <v>120</v>
+      </c>
+      <c r="E11" s="14">
+        <v>90</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>180</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="A12" s="13">
+        <v>46250</v>
+      </c>
+      <c r="B12" s="14">
+        <v>600</v>
+      </c>
+      <c r="C12" s="14">
+        <v>30</v>
+      </c>
+      <c r="D12" s="14">
+        <v>180</v>
+      </c>
+      <c r="E12" s="14">
+        <v>90</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>180</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>

</xml_diff>

<commit_message>
Updated daily - routine 22-Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995982E9-309B-4B1E-89BE-1AB60C207563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F067DE3E-CF09-4249-984A-D1667A538AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">felt bit better today </t>
   </si>
 </sst>
 </file>
@@ -1600,26 +1603,50 @@
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B18" s="14">
+        <v>720</v>
+      </c>
+      <c r="C18" s="14">
+        <v>30</v>
+      </c>
+      <c r="D18" s="14">
+        <v>120</v>
+      </c>
+      <c r="E18" s="14">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>60</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>480</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>

</xml_diff>

<commit_message>
Updated daily-routine  26 Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C27AC76-BB9B-4270-8533-EB84495902CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9EE5EEA-064D-4C43-B7EB-FC60074CF873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -278,6 +278,12 @@
   </si>
   <si>
     <t>studied dbms</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>had a stomach ache</t>
   </si>
 </sst>
 </file>
@@ -1793,26 +1799,50 @@
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B22" s="14">
+        <v>600</v>
+      </c>
+      <c r="C22" s="14">
+        <v>0</v>
+      </c>
+      <c r="D22" s="14">
+        <v>0</v>
+      </c>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14">
+        <v>400</v>
+      </c>
+      <c r="G22" s="14">
+        <v>8</v>
+      </c>
+      <c r="H22" s="14">
+        <v>120</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>320</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
Updated daily-routine 27 Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9EE5EEA-064D-4C43-B7EB-FC60074CF873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821C9690-303B-4B33-A0DC-0326F8137A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>had a stomach ache</t>
+  </si>
+  <si>
+    <t>studied networking</t>
   </si>
 </sst>
 </file>
@@ -1845,26 +1848,50 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B23" s="14">
+        <v>600</v>
+      </c>
+      <c r="C23" s="14">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14">
+        <v>120</v>
+      </c>
+      <c r="E23" s="14">
+        <v>30</v>
+      </c>
+      <c r="F23" s="14">
+        <v>250</v>
+      </c>
+      <c r="G23" s="14">
+        <v>5</v>
+      </c>
+      <c r="H23" s="14">
+        <v>120</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>320</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>

</xml_diff>

<commit_message>
Updated Daily-routine 28 Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821C9690-303B-4B33-A0DC-0326F8137A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3D23AE-81BB-489B-B728-5DA3197258FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1894,26 +1894,50 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B24" s="14">
+        <v>480</v>
+      </c>
+      <c r="C24" s="14">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14">
+        <v>120</v>
+      </c>
+      <c r="E24" s="14">
+        <v>30</v>
+      </c>
+      <c r="F24" s="14">
+        <v>250</v>
+      </c>
+      <c r="G24" s="14">
+        <v>5</v>
+      </c>
+      <c r="H24" s="14">
+        <v>120</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1000</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>440</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>

</xml_diff>

<commit_message>
Updated daily-routine 29 Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3D23AE-81BB-489B-B728-5DA3197258FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615032D7-F3AE-466E-ADE8-7E5C9C80D54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1940,26 +1940,50 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+      <c r="A25" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B25" s="14">
+        <v>480</v>
+      </c>
+      <c r="C25" s="14">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14">
+        <v>60</v>
+      </c>
+      <c r="E25" s="14">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14">
+        <v>60</v>
+      </c>
+      <c r="G25" s="14">
+        <v>1</v>
+      </c>
+      <c r="H25" s="14">
+        <v>240</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
+        <v>600</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>

</xml_diff>

<commit_message>
Updated daily- routine 30-Aug
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615032D7-F3AE-466E-ADE8-7E5C9C80D54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E176CC47-120F-4EAF-B7C7-D09762033E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1986,26 +1986,50 @@
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+      <c r="A26" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B26" s="14">
+        <v>540</v>
+      </c>
+      <c r="C26" s="14">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14">
+        <v>180</v>
+      </c>
+      <c r="E26" s="14">
+        <v>60</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14">
+        <v>120</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>540</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>

</xml_diff>

<commit_message>
Updated daily-routine 1-September -2026
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FC3CCF-018A-4C58-9148-B94EB43FFF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67300AAA-2F4F-42FE-B5AD-5EEA09D702B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2078,26 +2078,50 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B28" s="14">
+        <v>540</v>
+      </c>
+      <c r="C28" s="14">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14">
+        <v>120</v>
+      </c>
+      <c r="E28" s="14">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14">
+        <v>400</v>
+      </c>
+      <c r="G28" s="14">
+        <v>8</v>
+      </c>
+      <c r="H28" s="14">
+        <v>120</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>230</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>

</xml_diff>

<commit_message>
Updated daily routine 11-sep
</commit_message>
<xml_diff>
--- a/Daily_Routine_.xlsx
+++ b/Daily_Routine_.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artim\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MCA\Semester 1\python\My data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935947F3-7A14-4220-8323-A066C8C5C8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC8BF32-4765-4E28-B3ED-738FF28C0602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>felt low after the last class</t>
+  </si>
+  <si>
+    <t>Neutral</t>
   </si>
 </sst>
 </file>
@@ -2547,26 +2550,50 @@
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+      <c r="A38" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B38" s="14">
+        <v>480</v>
+      </c>
+      <c r="C38" s="14">
+        <v>0</v>
+      </c>
+      <c r="D38" s="14">
+        <v>120</v>
+      </c>
+      <c r="E38" s="14">
+        <v>30</v>
+      </c>
+      <c r="F38" s="14">
+        <v>300</v>
+      </c>
+      <c r="G38" s="14">
+        <v>6</v>
+      </c>
+      <c r="H38" s="14">
+        <v>120</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>

</xml_diff>